<commit_message>
Update weekly ranking [2026-03-04]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -26,6 +26,7 @@
     <sheet name="magapoke_2026-02-11" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="magapoke_2026-02-18" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="magapoke_2026-02-25" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="magapoke_2026-03-04" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6259,6 +6260,512 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>黒月のイェルクナハト</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ドリーム☆ジャンボ☆ガール</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>【爆アド】生まれた直後から最強悪霊と脳内バトルしてたら魔力量が測定可能域を超えてました〜悪憑の子の謙虚な覇道〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>K-9~警視庁公安部公安第9課異能対策係~</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ハードワーカー中田</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ペンの夢に紅をさす</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>追放されなかった男　～二度目の人生は土下座から始まりました～</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>怨霊日和</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ルックスＹを選んでしまいました 〜やり込んでいるゲームに転生したはずなのに、未実装のガチャで攻略をすることになった件〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>春くらり</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>白鳥運子は31画</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>MYS</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>限界集落を脱村した錬金術士、都会で"最強"なのがバレまくる。～老害どもにはいい加減愛想が尽きました～</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>わが投資術　市場は誰に微笑むか</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>異世界グルメで成り上がり無双～山に追放されたので、のんびりキャンプを楽しんでいたらいつの間にか強くなっていて、王侯貴族や実力者たちが俺を放っておいてくれません。一方、俺を追放した貴族たちは破滅が始まる～</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>屋根の下のアルテミス</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>せいぶつ部の田辺くん</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ともだちづくり</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>鳴るさんだぁ</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>じゅーくぼっくす</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ハプスブルク家の華麗なる受難</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>皇女転生　～伝説の大魔導士（♂）、姫騎士となりて伝説の令嬢騎士団を作り無双する～</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>明智ナンバーワン</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>平成転生</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>君が監督！</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ch登録お願いします！</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>歪みの虜</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>人生逆転ダンジョン</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>GURU</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>花子狩り</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>邪目さんは邪神です</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>ナマイキ旭ちゃんをわからせたい</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>白銀のキュイジーヌ～明治外交官の料理人～</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>宇曽田みのりの代用料理</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>眠れる森のレガ</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>JK Biker</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>永久のユウグレ</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>イエティ、とある日々</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>きゃわるり方程式</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-03-11]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -27,6 +27,7 @@
     <sheet name="magapoke_2026-02-18" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="magapoke_2026-02-25" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="magapoke_2026-03-04" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="magapoke_2026-03-11" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6766,6 +6767,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>黒月のイェルクナハト</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ドリーム☆ジャンボ☆ガール</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>【爆アド】生まれた直後から最強悪霊と脳内バトルしてたら魔力量が測定可能域を超えてました〜悪憑の子の謙虚な覇道〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>K-9~警視庁公安部公安第9課異能対策係~</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ハードワーカー中田</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>せいぶつ部の田辺くん</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>白鳥運子は31画</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ルックスＹを選んでしまいました 〜やり込んでいるゲームに転生したはずなのに、未実装のガチャで攻略をすることになった件〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ペンの夢に紅をさす</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>怨霊日和</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>皇女転生　～伝説の大魔導士（♂）、姫騎士となりて伝説の令嬢騎士団を作り無双する～</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>春くらり</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>解除師カンナの魔術録</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>屋根の下のアルテミス</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>MYS</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>異世界グルメで成り上がり無双～山に追放されたので、のんびりキャンプを楽しんでいたらいつの間にか強くなっていて、王侯貴族や実力者たちが俺を放っておいてくれません。一方、俺を追放した貴族たちは破滅が始まる～</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-03-18]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -28,6 +28,7 @@
     <sheet name="magapoke_2026-02-25" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="magapoke_2026-03-04" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="magapoke_2026-03-11" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="magapoke_2026-03-18" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7043,6 +7044,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ドリーム☆ジャンボ☆ガール</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>【爆アド】生まれた直後から最強悪霊と脳内バトルしてたら魔力量が測定可能域を超えてました〜悪憑の子の謙虚な覇道〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ハードワーカー中田</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>K-9~警視庁公安部公安第9課異能対策係~</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>せいぶつ部の田辺くん</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ペンの夢に紅をさす</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>追放されなかった男　～二度目の人生は土下座から始まりました～</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ルックスＹを選んでしまいました 〜やり込んでいるゲームに転生したはずなのに、未実装のガチャで攻略をすることになった件〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>黒月のイェルクナハト</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>眠れる森のレガ</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>白鳥運子は31画</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>屋根の下のアルテミス</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>わが投資術　市場は誰に微笑むか</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>限界集落を脱村した錬金術士、都会で"最強"なのがバレまくる。～老害どもにはいい加減愛想が尽きました～</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>異世界グルメで成り上がり無双～山に追放されたので、のんびりキャンプを楽しんでいたらいつの間にか強くなっていて、王侯貴族や実力者たちが俺を放っておいてくれません。一方、俺を追放した貴族たちは破滅が始まる～</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-03-25]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -29,6 +29,7 @@
     <sheet name="magapoke_2026-03-04" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="magapoke_2026-03-11" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="magapoke_2026-03-18" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="magapoke_2026-03-25" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7320,6 +7321,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>黒月のイェルクナハト</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>【爆アド】生まれた直後から最強悪霊と脳内バトルしてたら魔力量が測定可能域を超えてました〜悪憑の子の謙虚な覇道〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>せいぶつ部の田辺くん</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ともだちづくり</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ペンの夢に紅をさす</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ルックスＹを選んでしまいました 〜やり込んでいるゲームに転生したはずなのに、未実装のガチャで攻略をすることになった件〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ドリーム☆ジャンボ☆ガール</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>白鳥運子は31画</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>屋根の下のアルテミス</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>限界集落を脱村した錬金術士、都会で"最強"なのがバレまくる。～老害どもにはいい加減愛想が尽きました～</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>わが投資術　市場は誰に微笑むか</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>異世界グルメで成り上がり無双～山に追放されたので、のんびりキャンプを楽しんでいたらいつの間にか強くなっていて、王侯貴族や実力者たちが俺を放っておいてくれません。一方、俺を追放した貴族たちは破滅が始まる～</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>K-9~警視庁公安部公安第9課異能対策係~</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>そして刹那は繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>君が監督！</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-04-01]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -30,6 +30,7 @@
     <sheet name="magapoke_2026-03-11" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="magapoke_2026-03-18" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="magapoke_2026-03-25" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="magapoke_2026-04-01" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7597,6 +7598,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>まじイヌ</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>【爆アド】生まれた直後から最強悪霊と脳内バトルしてたら魔力量が測定可能域を超えてました〜悪憑の子の謙虚な覇道〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ペンの夢に紅をさす</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>黒月のイェルクナハト</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ドリーム☆ジャンボ☆ガール</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>K-9~警視庁公安部公安第9課異能対策係~</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>せいぶつ部の田辺くん</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ルックスＹを選んでしまいました 〜やり込んでいるゲームに転生したはずなのに、未実装のガチャで攻略をすることになった件〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>白鳥運子は31画</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>わが投資術　市場は誰に微笑むか</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>皇女転生　～伝説の大魔導士（♂）、姫騎士となりて伝説の令嬢騎士団を作り無双する～</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>限界集落を脱村した錬金術士、都会で"最強"なのがバレまくる。～老害どもにはいい加減愛想が尽きました～</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>そして刹那は繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>異世界グルメで成り上がり無双～山に追放されたので、のんびりキャンプを楽しんでいたらいつの間にか強くなっていて、王侯貴族や実力者たちが俺を放っておいてくれません。一方、俺を追放した貴族たちは破滅が始まる～</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>屋根の下のアルテミス</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>君が監督！</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-04-08]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -31,6 +31,7 @@
     <sheet name="magapoke_2026-03-18" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="magapoke_2026-03-25" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="magapoke_2026-04-01" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="magapoke_2026-04-08" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7874,6 +7875,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>K-9~警視庁公安部公安第9課異能対策係~</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>黒月のイェルクナハト</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ドリーム☆ジャンボ☆ガール</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>【爆アド】生まれた直後から最強悪霊と脳内バトルしてたら魔力量が測定可能域を超えてました〜悪憑の子の謙虚な覇道〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>せいぶつ部の田辺くん</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>白鳥運子は31画</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ともだちづくり</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ペンの夢に紅をさす</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>まじイヌ</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>屋根の下のアルテミス</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>限界集落を脱村した錬金術士、都会で"最強"なのがバレまくる。～老害どもにはいい加減愛想が尽きました～</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>わが投資術　市場は誰に微笑むか</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>追放されなかった男　～二度目の人生は土下座から始まりました～</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>平成転生</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>そして刹那は繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>異世界グルメで成り上がり無双～山に追放されたので、のんびりキャンプを楽しんでいたらいつの間にか強くなっていて、王侯貴族や実力者たちが俺を放っておいてくれません。一方、俺を追放した貴族たちは破滅が始まる～</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-04-15]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -32,6 +32,7 @@
     <sheet name="magapoke_2026-03-25" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="magapoke_2026-04-01" sheetId="24" state="visible" r:id="rId24"/>
     <sheet name="magapoke_2026-04-08" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="magapoke_2026-04-15" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -8151,6 +8152,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ドリーム☆ジャンボ☆ガール</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>【爆アド】生まれた直後から最強悪霊と脳内バトルしてたら魔力量が測定可能域を超えてました〜悪憑の子の謙虚な覇道〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>K-9~警視庁公安部公安第9課異能対策係~</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>せいぶつ部の田辺くん</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ぎるてぃらいぶらり</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ペンの夢に紅をさす</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>白鳥運子は31画</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>皇女転生　～伝説の大魔導士（♂）、姫騎士となりて伝説の令嬢騎士団を作り無双する～</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>そして刹那は繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>人生逆転ダンジョン</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>わが投資術　市場は誰に微笑むか</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>限界集落を脱村した錬金術士、都会で"最強"なのがバレまくる。～老害どもにはいい加減愛想が尽きました～</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>人狼とエルフ</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ch登録お願いします！</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>転生したらウイニングイレブンだった件</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-04-22]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -33,6 +33,7 @@
     <sheet name="magapoke_2026-04-01" sheetId="24" state="visible" r:id="rId24"/>
     <sheet name="magapoke_2026-04-08" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="magapoke_2026-04-15" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="magapoke_2026-04-22" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -8428,6 +8429,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ジャンクシュート</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ドリーム☆ジャンボ☆ガール</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>【爆アド】生まれた直後から最強悪霊と脳内バトルしてたら魔力量が測定可能域を超えてました〜悪憑の子の謙虚な覇道〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>せいぶつ部の田辺くん</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ともだちづくり</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ペンの夢に紅をさす</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>堕天使ちゃんはがんばれない</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ぎるてぃらいぶらり</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>男子高校生のススメ</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>眠れる森のレガ</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>白鳥運子は31画</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>限界集落を脱村した錬金術士、都会で"最強"なのがバレまくる。～老害どもにはいい加減愛想が尽きました～</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>そして刹那は繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>わが投資術　市場は誰に微笑むか</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>麗しババアは孫が欲しい！</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-04-29]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -34,6 +34,7 @@
     <sheet name="magapoke_2026-04-08" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="magapoke_2026-04-15" sheetId="26" state="visible" r:id="rId26"/>
     <sheet name="magapoke_2026-04-22" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="magapoke_2026-04-29" sheetId="28" state="visible" r:id="rId28"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -8705,6 +8706,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ジャンクシュート</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ドリーム☆ジャンボ☆ガール</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>【爆アド】生まれた直後から最強悪霊と脳内バトルしてたら魔力量が測定可能域を超えてました〜悪憑の子の謙虚な覇道〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ペンの夢に紅をさす</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>白鳥運子は31画</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>男子高校生のススメ</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>わが投資術　市場は誰に微笑むか</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>堕天使ちゃんはがんばれない</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>そして刹那は繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>麗しババアは孫が欲しい！</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>異世界グルメで成り上がり無双～山に追放されたので、のんびりキャンプを楽しんでいたらいつの間にか強くなっていて、王侯貴族や実力者たちが俺を放っておいてくれません。一方、俺を追放した貴族たちは破滅が始まる～</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>せいぶつ部の田辺くん</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>歪みの虜</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>君が監督！</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>転生したらウイニングイレブンだった件</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-05-06]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -35,6 +35,7 @@
     <sheet name="magapoke_2026-04-15" sheetId="26" state="visible" r:id="rId26"/>
     <sheet name="magapoke_2026-04-22" sheetId="27" state="visible" r:id="rId27"/>
     <sheet name="magapoke_2026-04-29" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="magapoke_2026-05-06" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -8982,6 +8983,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ジャンクシュート</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>【爆アド】生まれた直後から最強悪霊と脳内バトルしてたら魔力量が測定可能域を超えてました〜悪憑の子の謙虚な覇道〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ドリーム☆ジャンボ☆ガール</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ペンの夢に紅をさす</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>白鳥運子は31画</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>皇女転生　～伝説の大魔導士（♂）、姫騎士となりて伝説の令嬢騎士団を作り無双する～</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>そして刹那は繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>君が監督！</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>限界集落を脱村した錬金術士、都会で"最強"なのがバレまくる。～老害どもにはいい加減愛想が尽きました～</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>堕天使ちゃんはがんばれない</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ロブレイブ</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>GURU</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>異世界グルメで成り上がり無双～山に追放されたので、のんびりキャンプを楽しんでいたらいつの間にか強くなっていて、王侯貴族や実力者たちが俺を放っておいてくれません。一方、俺を追放した貴族たちは破滅が始まる～</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>歪みの虜</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>平成転生</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-05-13]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -36,6 +36,7 @@
     <sheet name="magapoke_2026-04-22" sheetId="27" state="visible" r:id="rId27"/>
     <sheet name="magapoke_2026-04-29" sheetId="28" state="visible" r:id="rId28"/>
     <sheet name="magapoke_2026-05-06" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="magapoke_2026-05-13" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9705,6 +9706,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>りりむホリック</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ドリーム☆ジャンボ☆ガール</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>【爆アド】生まれた直後から最強悪霊と脳内バトルしてたら魔力量が測定可能域を超えてました〜悪憑の子の謙虚な覇道〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ジャンクシュート</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ペンの夢に紅をさす</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>白鳥運子は31画</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>そして刹那は繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>シロナガス島への帰還</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>麗しババアは孫が欲しい！</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>堕天使ちゃんはがんばれない</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>異世界グルメで成り上がり無双～山に追放されたので、のんびりキャンプを楽しんでいたらいつの間にか強くなっていて、王侯貴族や実力者たちが俺を放っておいてくれません。一方、俺を追放した貴族たちは破滅が始まる～</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ロブレイブ</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ハプスブルク家の華麗なる受難</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>人狼とエルフ</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>歪みの虜</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-05-20]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -37,6 +37,7 @@
     <sheet name="magapoke_2026-04-29" sheetId="28" state="visible" r:id="rId28"/>
     <sheet name="magapoke_2026-05-06" sheetId="29" state="visible" r:id="rId29"/>
     <sheet name="magapoke_2026-05-13" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="magapoke_2026-05-20" sheetId="31" state="visible" r:id="rId31"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9982,6 +9983,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>りりむホリック</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>【爆アド】生まれた直後から最強悪霊と脳内バトルしてたら魔力量が測定可能域を超えてました〜悪憑の子の謙虚な覇道〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>そして刹那は繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ジャンクシュート</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ドリーム☆ジャンボ☆ガール</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>君が監督！</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>眠れる森のレガ</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>白鳥運子は31画</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>皇女転生　～伝説の大魔導士（♂）、姫騎士となりて伝説の令嬢騎士団を作り無双する～</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>堕天使ちゃんはがんばれない</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>麗しババアは孫が欲しい！</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ロブレイブ</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ペンの夢に紅をさす</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ナマイキ旭ちゃんをわからせたい</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>シロナガス島への帰還</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-05-27]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -38,6 +38,7 @@
     <sheet name="magapoke_2026-05-06" sheetId="29" state="visible" r:id="rId29"/>
     <sheet name="magapoke_2026-05-13" sheetId="30" state="visible" r:id="rId30"/>
     <sheet name="magapoke_2026-05-20" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="magapoke_2026-05-27" sheetId="32" state="visible" r:id="rId32"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -10259,6 +10260,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>りりむホリック</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>【爆アド】生まれた直後から最強悪霊と脳内バトルしてたら魔力量が測定可能域を超えてました〜悪憑の子の謙虚な覇道〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ジャンクシュート</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ペンの夢に紅をさす</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ドリーム☆ジャンボ☆ガール</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>おれは美少女VTuber</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>そして刹那は繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>麗しババアは孫が欲しい！</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>異世界グルメで成り上がり無双～山に追放されたので、のんびりキャンプを楽しんでいたらいつの間にか強くなっていて、王侯貴族や実力者たちが俺を放っておいてくれません。一方、俺を追放した貴族たちは破滅が始まる～</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>君が監督！</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ロブレイブ</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>白鳥運子は31画</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>皇女転生　～伝説の大魔導士（♂）、姫騎士となりて伝説の令嬢騎士団を作り無双する～</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>堕天使ちゃんはがんばれない</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>宇曽田みのりの代用料理</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-06-03]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -39,6 +39,7 @@
     <sheet name="magapoke_2026-05-13" sheetId="30" state="visible" r:id="rId30"/>
     <sheet name="magapoke_2026-05-20" sheetId="31" state="visible" r:id="rId31"/>
     <sheet name="magapoke_2026-05-27" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="magapoke_2026-06-03" sheetId="33" state="visible" r:id="rId33"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -10536,6 +10537,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>【爆アド】生まれた直後から最強悪霊と脳内バトルしてたら魔力量が測定可能域を超えてました〜悪憑の子の謙虚な覇道〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>りりむホリック</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ジャンクシュート</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ペンの夢に紅をさす</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>白鳥運子は31画</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>そして刹那は繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>皇女転生　～伝説の大魔導士（♂）、姫騎士となりて伝説の令嬢騎士団を作り無双する～</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>堕天使ちゃんはがんばれない</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>異世界グルメで成り上がり無双～山に追放されたので、のんびりキャンプを楽しんでいたらいつの間にか強くなっていて、王侯貴族や実力者たちが俺を放っておいてくれません。一方、俺を追放した貴族たちは破滅が始まる～</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>宇曽田みのりの代用料理</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>闇覚醒して主人公にボコされるかませ犬に憑依したが原作と違いすぎて戸惑ってる</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>君が監督！</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>麗しババアは孫が欲しい！</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ロブレイブ</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>じゅーくぼっくす</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-06-10]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -40,6 +40,7 @@
     <sheet name="magapoke_2026-05-20" sheetId="31" state="visible" r:id="rId31"/>
     <sheet name="magapoke_2026-05-27" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="magapoke_2026-06-03" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="magapoke_2026-06-10" sheetId="34" state="visible" r:id="rId34"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -10813,6 +10814,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>千仙戦記</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ジャンクシュート</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ダンジョンの測量士～地図で無双するダンジョン攻略～</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>アイ・ヘイ・チュー</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>【爆アド】生まれた直後から最強悪霊と脳内バトルしてたら魔力量が測定可能域を超えてました〜悪憑の子の謙虚な覇道〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ペンの夢に紅をさす</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>りりむホリック</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>麗しババアは孫が欲しい！</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>シロナガス島への帰還</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>人狼とエルフ</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ロブレイブ</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>白鳥運子は31画</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ゲーム開始前に死ぬモブ悪役皇子に転生した俺　～推しヒロインの妹と幸せになるために最弱魔法【闇刃】を過剰な努力で極め抜いたら、最強のぶっ壊れ性能と化していた件～</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>おれは美少女VTuber</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>闇覚醒して主人公にボコされるかませ犬に憑依したが原作と違いすぎて戸惑ってる</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>